<commit_message>
feat: incorporar compra de empanadas (Joaquín) y comensal Franklin
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,13 +59,19 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="002563EB"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00DC2626"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="006B7280"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -127,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +159,7 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -519,10 +526,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -536,7 +543,13 @@
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,167 +585,157 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Total cuarta compra (Joaquín)</t>
+          <t>Total cuarta compra (Joaquín - Pan choripán)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
         <v>5570</v>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Total quinta compra (Joaquín - Empanadas)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46250</v>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Chorizo</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Lomo Liso</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Lomo vetado</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Costillar Chileno</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Costillar cerdo</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Trutro</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Pechuga</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Carbón</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Pan Choripán</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Trigo Mote (1kg)</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Huesillos (1kg)</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Chancaca y Azúcar</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Restante</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Pino (1a Empanada)</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Pino (2a Empanada)</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Mechada</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Camarón Queso</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Queso</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Napolitana</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
         <is>
           <t>Total Fila</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Primera compra (Ignacio)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>14670</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>21226</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>19560</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>19238</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>14957</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>2490</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>10990</v>
-      </c>
-      <c r="M7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>19120</v>
-      </c>
-      <c r="O7" s="5">
-        <f>SUM(B7:N7)</f>
-        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Segunda compra (Ignacio)</t>
+          <t>Primera compra (Ignacio)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>4890</v>
+        <v>14670</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0</v>
+        <v>21226</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>33693</v>
+        <v>19560</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0</v>
+        <v>19238</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>14957</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>16353</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6205</v>
+        <v>0</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>0</v>
@@ -741,36 +744,54 @@
         <v>0</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0</v>
+        <v>2490</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>0</v>
+        <v>10990</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="5">
-        <f>SUM(B8:N8)</f>
+        <v>19120</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="5">
+        <f>SUM(B8:T8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Tercera compra (Mindy)</t>
+          <t>Segunda compra (Ignacio)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>0</v>
+        <v>4890</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0</v>
+        <v>33693</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>0</v>
@@ -779,13 +800,13 @@
         <v>0</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>16353</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0</v>
+        <v>6205</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>8400</v>
+        <v>0</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>0</v>
@@ -797,20 +818,38 @@
         <v>0</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>3390</v>
+        <v>0</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="5">
-        <f>SUM(B9:N9)</f>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="5">
+        <f>SUM(B9:T9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Cuarta compra (Joaquín)</t>
+          <t>Tercera compra (Mindy)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -835,10 +874,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0</v>
+        <v>8400</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5570</v>
+        <v>0</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>0</v>
@@ -847,76 +886,254 @@
         <v>0</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0</v>
+        <v>3390</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O10" s="5">
-        <f>SUM(B10:N10)</f>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="5">
+        <f>SUM(B10:T10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
+          <t>Cuarta compra (Joaquín)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>5570</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="5">
+        <f>SUM(B11:T11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Quinta compra (Joaquín - Empanadas)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>17500</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>6000</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>2250</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>2500</v>
+      </c>
+      <c r="U12" s="5">
+        <f>SUM(B12:T12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B11" s="5">
-        <f>SUM(B7:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>SUM(C7:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>SUM(D7:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>SUM(E7:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="5">
-        <f>SUM(F7:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="5">
-        <f>SUM(G7:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="5">
-        <f>SUM(H7:H10)</f>
-        <v/>
-      </c>
-      <c r="I11" s="5">
-        <f>SUM(I7:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="5">
-        <f>SUM(J7:J10)</f>
-        <v/>
-      </c>
-      <c r="K11" s="5">
-        <f>SUM(K7:K10)</f>
-        <v/>
-      </c>
-      <c r="L11" s="5">
-        <f>SUM(L7:L10)</f>
-        <v/>
-      </c>
-      <c r="M11" s="5">
-        <f>SUM(M7:M10)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5">
-        <f>SUM(N7:N10)</f>
-        <v/>
-      </c>
-      <c r="O11" s="6">
-        <f>SUM(O7:O10)</f>
+      <c r="B13" s="5">
+        <f>SUM(B8:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>SUM(C8:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>SUM(D8:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>SUM(E8:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>SUM(F8:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>SUM(G8:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>SUM(H8:H12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="5">
+        <f>SUM(I8:I12)</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>SUM(J8:J12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>SUM(K8:K12)</f>
+        <v/>
+      </c>
+      <c r="L13" s="5">
+        <f>SUM(L8:L12)</f>
+        <v/>
+      </c>
+      <c r="M13" s="5">
+        <f>SUM(M8:M12)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5">
+        <f>SUM(N8:N12)</f>
+        <v/>
+      </c>
+      <c r="O13" s="5">
+        <f>SUM(O8:O12)</f>
+        <v/>
+      </c>
+      <c r="P13" s="5">
+        <f>SUM(P8:P12)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="5">
+        <f>SUM(Q8:Q12)</f>
+        <v/>
+      </c>
+      <c r="R13" s="5">
+        <f>SUM(R8:R12)</f>
+        <v/>
+      </c>
+      <c r="S13" s="5">
+        <f>SUM(S8:S12)</f>
+        <v/>
+      </c>
+      <c r="T13" s="5">
+        <f>SUM(T8:T12)</f>
+        <v/>
+      </c>
+      <c r="U13" s="6">
+        <f>SUM(U8:U12)</f>
         <v/>
       </c>
     </row>
@@ -931,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -948,6 +1165,12 @@
     <col width="25" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1021,6 +1244,36 @@
           <t>Restante</t>
         </is>
       </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Pino (1a Empanada)</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Pino (2a Empanada)</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Mechada</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Camarón Queso</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Queso</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Napolitana</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1093,6 +1346,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P2" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1165,6 +1448,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S3" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1237,6 +1550,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -1309,6 +1652,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1381,6 +1754,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T6" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1453,6 +1856,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1525,6 +1958,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T8" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1597,6 +2060,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T9" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1669,6 +2162,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1741,6 +2264,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T11" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1813,6 +2366,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T12" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1885,6 +2468,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1957,6 +2570,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -2029,6 +2672,36 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -2101,63 +2774,219 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T16" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
+          <t>Franklin</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R17" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T17" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
           <t>Total Consumidores</t>
         </is>
       </c>
-      <c r="B17" s="9">
-        <f>COUNTIF(B2:B16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="C17" s="9">
-        <f>COUNTIF(C2:C16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="D17" s="9">
-        <f>COUNTIF(D2:D16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="E17" s="9">
-        <f>COUNTIF(E2:E16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="F17" s="9">
-        <f>COUNTIF(F2:F16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="G17" s="9">
-        <f>COUNTIF(G2:G16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="H17" s="9">
-        <f>COUNTIF(H2:H16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="I17" s="9">
-        <f>COUNTIF(I2:I16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="J17" s="9">
-        <f>COUNTIF(J2:J16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="K17" s="9">
-        <f>COUNTIF(K2:K16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="L17" s="9">
-        <f>COUNTIF(L2:L16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="M17" s="9">
-        <f>COUNTIF(M2:M16, "Sí")</f>
-        <v/>
-      </c>
-      <c r="N17" s="9">
-        <f>COUNTIF(N2:N16, "Sí")</f>
+      <c r="B18" s="9">
+        <f>COUNTIF(B2:B17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="C18" s="9">
+        <f>COUNTIF(C2:C17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="D18" s="9">
+        <f>COUNTIF(D2:D17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="E18" s="9">
+        <f>COUNTIF(E2:E17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="F18" s="9">
+        <f>COUNTIF(F2:F17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="G18" s="9">
+        <f>COUNTIF(G2:G17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="H18" s="9">
+        <f>COUNTIF(H2:H17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="I18" s="9">
+        <f>COUNTIF(I2:I17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="J18" s="9">
+        <f>COUNTIF(J2:J17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="K18" s="9">
+        <f>COUNTIF(K2:K17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="L18" s="9">
+        <f>COUNTIF(L2:L17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="M18" s="9">
+        <f>COUNTIF(M2:M17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="N18" s="9">
+        <f>COUNTIF(N2:N17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="O18" s="9">
+        <f>COUNTIF(O2:O17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="P18" s="9">
+        <f>COUNTIF(P2:P17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="9">
+        <f>COUNTIF(Q2:Q17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="R18" s="9">
+        <f>COUNTIF(R2:R17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="S18" s="9">
+        <f>COUNTIF(S2:S17, "Sí")</f>
+        <v/>
+      </c>
+      <c r="T18" s="9">
+        <f>COUNTIF(T2:T17, "Sí")</f>
         <v/>
       </c>
     </row>
@@ -2172,17 +3001,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="1169" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="1703" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2213,17 +3042,17 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Saldo Final a Transferir</t>
+          <t>Saldo a Liquidar</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Destinatario</t>
+          <t>Destinatario / Acción</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Estado Pago</t>
+          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -2234,7 +3063,7 @@
         </is>
       </c>
       <c r="B2" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B2="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C2="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D2="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E2="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F2="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G2="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H2="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I2="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J2="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K2="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L2="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M2="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N2="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B2="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C2="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D2="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E2="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F2="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G2="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H2="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I2="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J2="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K2="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L2="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M2="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N2="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O2="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P2="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q2="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R2="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S2="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T2="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C2" s="10">
@@ -2254,7 +3083,7 @@
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H2" s="12" t="inlineStr">
@@ -2270,7 +3099,7 @@
         </is>
       </c>
       <c r="B3" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B3="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C3="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D3="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E3="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F3="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G3="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H3="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I3="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J3="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K3="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L3="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M3="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N3="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B3="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C3="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D3="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E3="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F3="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G3="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H3="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I3="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J3="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K3="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L3="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M3="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N3="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O3="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P3="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q3="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R3="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S3="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T3="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C3" s="4" t="n">
@@ -2289,7 +3118,7 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
@@ -2305,7 +3134,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B4="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C4="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D4="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E4="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F4="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G4="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H4="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I4="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J4="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K4="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L4="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M4="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N4="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B4="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C4="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D4="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E4="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F4="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G4="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H4="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I4="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J4="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K4="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L4="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M4="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N4="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O4="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P4="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q4="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R4="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S4="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T4="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C4" s="10">
@@ -2317,20 +3146,20 @@
         <v/>
       </c>
       <c r="E4" s="4" t="n">
-        <v>5570</v>
-      </c>
-      <c r="F4" s="11">
-        <f>IF(D4-E4&gt;0, D4-E4, 0)</f>
+        <v>51820</v>
+      </c>
+      <c r="F4" s="13">
+        <f>E4-D4</f>
         <v/>
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Ignacio le transfiere (Saldo a favor)</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>A favor (Recibe)</t>
         </is>
       </c>
     </row>
@@ -2341,7 +3170,7 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B5="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C5="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D5="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E5="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F5="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G5="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H5="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I5="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J5="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K5="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L5="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M5="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N5="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B5="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C5="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D5="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E5="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F5="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G5="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H5="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I5="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J5="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K5="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L5="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M5="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N5="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O5="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P5="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q5="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R5="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S5="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T5="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C5" s="4" t="n">
@@ -2354,12 +3183,13 @@
       <c r="E5" s="4" t="n">
         <v>183392</v>
       </c>
-      <c r="F5" s="13" t="n">
-        <v>0</v>
+      <c r="F5" s="10">
+        <f>E5-B5</f>
+        <v/>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Organizador (Recibe)</t>
+          <t>Organizador (Recauda $193.121)</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -2375,7 +3205,7 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B6="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C6="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D6="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E6="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F6="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G6="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H6="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I6="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J6="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K6="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L6="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M6="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N6="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B6="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C6="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D6="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E6="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F6="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G6="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H6="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I6="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J6="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K6="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L6="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M6="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N6="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O6="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P6="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q6="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R6="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S6="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T6="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C6" s="14">
@@ -2388,7 +3218,7 @@
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -2409,7 +3239,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B7="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C7="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D7="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E7="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F7="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G7="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H7="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I7="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J7="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K7="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L7="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M7="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N7="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B7="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C7="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D7="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E7="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F7="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G7="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H7="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I7="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J7="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K7="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L7="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M7="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N7="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O7="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P7="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q7="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R7="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S7="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T7="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C7" s="10">
@@ -2429,7 +3259,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -2445,7 +3275,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B8="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C8="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D8="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E8="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F8="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G8="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H8="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I8="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J8="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K8="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L8="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M8="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N8="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B8="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C8="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D8="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E8="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F8="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G8="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H8="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I8="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J8="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K8="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L8="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M8="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N8="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O8="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P8="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q8="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R8="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S8="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T8="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C8" s="4" t="n">
@@ -2464,7 +3294,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
@@ -2480,7 +3310,7 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B9="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C9="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D9="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E9="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F9="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G9="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H9="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I9="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J9="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K9="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L9="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M9="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N9="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B9="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C9="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D9="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E9="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F9="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G9="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H9="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I9="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J9="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K9="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L9="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M9="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N9="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O9="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P9="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q9="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R9="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S9="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T9="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C9" s="10">
@@ -2500,7 +3330,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -2516,7 +3346,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B10="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C10="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D10="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E10="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F10="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G10="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H10="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I10="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J10="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K10="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L10="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M10="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N10="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B10="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C10="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D10="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E10="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F10="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G10="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H10="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I10="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J10="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K10="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L10="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M10="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N10="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O10="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P10="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q10="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R10="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S10="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T10="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C10" s="4" t="n">
@@ -2535,7 +3365,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -2551,7 +3381,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B11="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C11="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D11="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E11="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F11="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G11="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H11="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I11="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J11="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K11="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L11="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M11="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N11="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B11="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C11="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D11="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E11="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F11="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G11="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H11="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I11="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J11="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K11="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L11="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M11="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N11="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O11="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P11="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q11="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R11="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S11="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T11="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C11" s="4" t="n">
@@ -2570,7 +3400,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
@@ -2586,7 +3416,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B12="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C12="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D12="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E12="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F12="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G12="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H12="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I12="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J12="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K12="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L12="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M12="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N12="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B12="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C12="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D12="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E12="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F12="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G12="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H12="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I12="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J12="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K12="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L12="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M12="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N12="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O12="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P12="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q12="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R12="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S12="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T12="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C12" s="4" t="n">
@@ -2605,7 +3435,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -2621,7 +3451,7 @@
         </is>
       </c>
       <c r="B13" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B13="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C13="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D13="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E13="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F13="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G13="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H13="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I13="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J13="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K13="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L13="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M13="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N13="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B13="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C13="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D13="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E13="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F13="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G13="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H13="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I13="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J13="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K13="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L13="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M13="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N13="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O13="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P13="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q13="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R13="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S13="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T13="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C13" s="4" t="n">
@@ -2640,7 +3470,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -2656,7 +3486,7 @@
         </is>
       </c>
       <c r="B14" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B14="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C14="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D14="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E14="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F14="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G14="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H14="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I14="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J14="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K14="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L14="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M14="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N14="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B14="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C14="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D14="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E14="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F14="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G14="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H14="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I14="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J14="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K14="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L14="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M14="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N14="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O14="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P14="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q14="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R14="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S14="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T14="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C14" s="4" t="n">
@@ -2675,7 +3505,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -2691,7 +3521,7 @@
         </is>
       </c>
       <c r="B15" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B15="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C15="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D15="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E15="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F15="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G15="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H15="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I15="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J15="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K15="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L15="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M15="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N15="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B15="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C15="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D15="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E15="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F15="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G15="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H15="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I15="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J15="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K15="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L15="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M15="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N15="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O15="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P15="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q15="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R15="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S15="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T15="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C15" s="4" t="n">
@@ -2710,7 +3540,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -2726,7 +3556,7 @@
         </is>
       </c>
       <c r="B16" s="4">
-        <f>ROUND(IF('Consumo por Integrante'!B16="Sí", Compras!B$11 / 'Consumo por Integrante'!B$17, 0) + IF('Consumo por Integrante'!C16="Sí", Compras!C$11 / 'Consumo por Integrante'!C$17, 0) + IF('Consumo por Integrante'!D16="Sí", Compras!D$11 / 'Consumo por Integrante'!D$17, 0) + IF('Consumo por Integrante'!E16="Sí", Compras!E$11 / 'Consumo por Integrante'!E$17, 0) + IF('Consumo por Integrante'!F16="Sí", Compras!F$11 / 'Consumo por Integrante'!F$17, 0) + IF('Consumo por Integrante'!G16="Sí", Compras!G$11 / 'Consumo por Integrante'!G$17, 0) + IF('Consumo por Integrante'!H16="Sí", Compras!H$11 / 'Consumo por Integrante'!H$17, 0) + IF('Consumo por Integrante'!I16="Sí", Compras!I$11 / 'Consumo por Integrante'!I$17, 0) + IF('Consumo por Integrante'!J16="Sí", Compras!J$11 / 'Consumo por Integrante'!J$17, 0) + IF('Consumo por Integrante'!K16="Sí", Compras!K$11 / 'Consumo por Integrante'!K$17, 0) + IF('Consumo por Integrante'!L16="Sí", Compras!L$11 / 'Consumo por Integrante'!L$17, 0) + IF('Consumo por Integrante'!M16="Sí", Compras!M$11 / 'Consumo por Integrante'!M$17, 0) + IF('Consumo por Integrante'!N16="Sí", Compras!N$11 / 'Consumo por Integrante'!N$17, 0), 0)</f>
+        <f>ROUND(IF('Consumo por Integrante'!B16="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C16="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D16="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E16="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F16="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G16="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H16="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I16="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J16="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K16="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L16="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M16="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N16="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O16="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P16="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q16="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R16="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S16="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T16="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
       <c r="C16" s="4" t="n">
@@ -2745,7 +3575,7 @@
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Ignacio</t>
+          <t>Transfiere a Ignacio</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
@@ -2757,31 +3587,70 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Total Recaudado</t>
-        </is>
-      </c>
-      <c r="B17" s="6">
-        <f>SUM(B2:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="6">
-        <f>SUM(C2:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="6">
-        <f>SUM(D2:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="6">
-        <f>SUM(E2:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="15">
-        <f>SUM(F2:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+          <t>Franklin</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f>ROUND(IF('Consumo por Integrante'!B17="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C17="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D17="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E17="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F17="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G17="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H17="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I17="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J17="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K17="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L17="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M17="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N17="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O17="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P17="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q17="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R17="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S17="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T17="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
+        <v/>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
+        <f>B17+C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11">
+        <f>IF(D17-E17&gt;0, D17-E17, 0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Transfiere a Ignacio</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Totales</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>SUM(E2:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="16">
+        <f>SUMIF(G2:G17, "Transfiere a Ignacio", F2:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>Total Recaudado por Ignacio</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: ajustar textos tarjetas Quena/Joaquin/Mindy/Ignacio y bloquear clics en estado
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -1686,7 +1686,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Kena</t>
+          <t>Quena</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -3006,7 +3006,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="1703" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Aporte Cuota Kena (1/4)</t>
+          <t>Aporte Cuota Quena (1/4)</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -3201,7 +3201,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Kena</t>
+          <t>Quena</t>
         </is>
       </c>
       <c r="B6" s="4">

</xml_diff>

<commit_message>
fix: corregir nombre de Miriam a Myriam
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -2400,7 +2400,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Miriam</t>
+          <t>Myriam</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -3447,7 +3447,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Miriam</t>
+          <t>Myriam</t>
         </is>
       </c>
       <c r="B13" s="4">

</xml_diff>

<commit_message>
fix: excluir a Myriam y Abuelo Coni de mote, huesillos y chancaca/azucar
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -2448,19 +2448,19 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L13" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -2550,19 +2550,19 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: registrar pagos de Pamela, Cote y Franklin y habilitar alternancia rapida
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="002563EB"/>
       <sz val="11"/>
     </font>
@@ -72,6 +78,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="006B7280"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00991B1B"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -133,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,9 +168,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -3086,9 +3100,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3121,9 +3135,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3162,7 @@
       <c r="E4" s="4" t="n">
         <v>51820</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="14">
         <f>E4-D4</f>
         <v/>
       </c>
@@ -3208,7 +3222,7 @@
         <f>ROUND(IF('Consumo por Integrante'!B6="Sí", Compras!B$13 / 'Consumo por Integrante'!B$18, 0) + IF('Consumo por Integrante'!C6="Sí", Compras!C$13 / 'Consumo por Integrante'!C$18, 0) + IF('Consumo por Integrante'!D6="Sí", Compras!D$13 / 'Consumo por Integrante'!D$18, 0) + IF('Consumo por Integrante'!E6="Sí", Compras!E$13 / 'Consumo por Integrante'!E$18, 0) + IF('Consumo por Integrante'!F6="Sí", Compras!F$13 / 'Consumo por Integrante'!F$18, 0) + IF('Consumo por Integrante'!G6="Sí", Compras!G$13 / 'Consumo por Integrante'!G$18, 0) + IF('Consumo por Integrante'!H6="Sí", Compras!H$13 / 'Consumo por Integrante'!H$18, 0) + IF('Consumo por Integrante'!I6="Sí", Compras!I$13 / 'Consumo por Integrante'!I$18, 0) + IF('Consumo por Integrante'!J6="Sí", Compras!J$13 / 'Consumo por Integrante'!J$18, 0) + IF('Consumo por Integrante'!K6="Sí", Compras!K$13 / 'Consumo por Integrante'!K$18, 0) + IF('Consumo por Integrante'!L6="Sí", Compras!L$13 / 'Consumo por Integrante'!L$18, 0) + IF('Consumo por Integrante'!M6="Sí", Compras!M$13 / 'Consumo por Integrante'!M$18, 0) + IF('Consumo por Integrante'!N6="Sí", Compras!N$13 / 'Consumo por Integrante'!N$18, 0) + IF('Consumo por Integrante'!O6="Sí", Compras!O$13 / 'Consumo por Integrante'!O$18, 0) + IF('Consumo por Integrante'!P6="Sí", Compras!P$13 / 'Consumo por Integrante'!P$18, 0) + IF('Consumo por Integrante'!Q6="Sí", Compras!Q$13 / 'Consumo por Integrante'!Q$18, 0) + IF('Consumo por Integrante'!R6="Sí", Compras!R$13 / 'Consumo por Integrante'!R$18, 0) + IF('Consumo por Integrante'!S6="Sí", Compras!S$13 / 'Consumo por Integrante'!S$18, 0) + IF('Consumo por Integrante'!T6="Sí", Compras!T$13 / 'Consumo por Integrante'!T$18, 0), 0)</f>
         <v/>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="15">
         <f>-B6</f>
         <v/>
       </c>
@@ -3218,7 +3232,7 @@
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="16" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -3262,7 +3276,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3297,7 +3311,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3333,7 +3347,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3368,7 +3382,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3403,7 +3417,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3438,7 +3452,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3473,7 +3487,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3508,7 +3522,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3543,7 +3557,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3578,7 +3592,7 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -3613,9 +3627,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3655,7 @@
         <f>SUM(E2:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="17">
         <f>SUMIF(G2:G17, "Transfiere a Ignacio", F2:F17)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: registrar pagos de Mauri, Mindy, Gustavo, Monse, Papa Mauri y Mama Mauri
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -3311,9 +3311,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3347,9 +3347,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3382,9 +3382,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3417,9 +3417,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3557,9 +3557,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3592,9 +3592,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: registrar pago de Ale
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -3276,9 +3276,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: registrar liquidacion de Joaquin y cuota 100% cubierta de Quena
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,12 +72,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00DC2626"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="006B7280"/>
       <sz val="11"/>
     </font>
     <font>
@@ -144,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,7 +167,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -3025,7 +3018,7 @@
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="41" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3171,9 +3164,9 @@
           <t>Ignacio le transfiere (Saldo a favor)</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>A favor (Recibe)</t>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Liquidado</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3225,7 @@
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="12" t="inlineStr">
@@ -3240,9 +3233,9 @@
           <t>Cubierto por familiares</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>Cubierto</t>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Cubierto (100%)</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3648,7 @@
         <f>SUM(E2:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="17">
+      <c r="F18" s="16">
         <f>SUMIF(G2:G17, "Transfiere a Ignacio", F2:F17)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: registrar pagos de Coni, Myriam y Abuelo Coni (16/16 recaudado)
</commit_message>
<xml_diff>
--- a/Cuentas Fiestas Patrias.xlsx
+++ b/Cuentas Fiestas Patrias.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,11 +72,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00DC2626"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00991B1B"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -3445,9 +3440,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3480,9 +3475,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>
@@ -3515,9 +3510,9 @@
           <t>Transfiere a Ignacio</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Pagado</t>
         </is>
       </c>
     </row>

</xml_diff>